<commit_message>
전 4개 데이터셋 void 검토 + False OK 감도 논증 (PhaseC)
TEST·TB500M·43런까지 확인 — 모두 같은 웨이퍼(126173086.17). void는 전량
Q<0.9 undersize 아티팩트(최대18.8%), Q정상(kV60)=void 0 → 웨이퍼 void-free.
0.1% threshold 아이디어: 검출 방향은 타당(0.1%잡으면 8%는 쉬움)하나 진짜
void 부재·나쁜조건 감도·오차 2/N 규모차로 수치대입 불가. False OK=감도상
낮음·미검증, 소형 진짜 void 1개면 확정.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEDPo1aa2m4Ui6JuqiXEbY
</commit_message>
<xml_diff>
--- a/공정모델링/2차_void정확도_DOE.xlsx
+++ b/공정모델링/2차_void정확도_DOE.xlsx
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -84,6 +84,15 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1704,7 +1713,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>→ 안전창: kV≤60(또는 정점) + R을 극단(0.35·0.65)으로 몰지 않기. 운영점 kV60·R0.5 = 완전 청정.</t>
@@ -2256,7 +2264,6 @@
       <c r="I15" t="n">
         <v>2</v>
       </c>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2292,7 +2299,6 @@
       <c r="I16" t="n">
         <v>3</v>
       </c>
-      <c r="L16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2308,34 +2314,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PhaseC — False OK(진짜 void 미검출) : 보류</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>PhaseC — False OK(진짜 void 미검출): 전 데이터셋 검토 결과</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>가장 중요한 오류(진짜 불량을 OK로 놓침)는 '진짜 void가 있는 샘플'이 있어야만 검증된다. 현재 2자재·웨이퍼는 void≈0(있는 건 전부 kV62 아티팩트)이라 검증 불가. → 불량 웨이퍼 또는 인위 void 샘플 확보 시 진행. 그 전까지 'False OK 미검증'을 모델 한계로 명시.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>■ 4개 데이터셋(DOE·TB500M·TEST·43런) 전수 확인 — 모두 같은 웨이퍼(126173086.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>void는 전량 Q_dia&lt;0.9(undersize) 조건의 아티팩트. void%가 undersize 정도에 비례(Q0.88→18.7%). Q정상(kV60·Q≈0.98)에선 void=0(예외: F32 3/2988·≤1%, 노이즈 추정). → 이 웨이퍼는 실제로 void가 없다.</t>
+        </is>
+      </c>
+    </row>
     <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>■ '0.1% threshold로 계산해 8%에 적용' 검토</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>방향은 타당: 시스템이 0.1%(≈1.6px)를 (아티팩트로라도) 잡으면 8% void(≈14.7px)는 훨씬 쉽게 잡음 → 감도부족으로 8% 놓칠(False OK) 가능성 낮음. 한계 3: ①진짜 void가 0.1%조차 없어 시험 대상 없음 ②그 감도는 나쁜조건(kV62)에서 본 것, 운영조건(kV60) 감도는 미실측 ③오차는 2/N이라 0.1%(오차125%)와 8%(오차13.6%)는 규모가 달라 수치 대입 불가(검출 여부에만 방향 적용).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>■ 결론</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>False OK 위험 = 감도상 낮음, 그러나 미검증(진짜 void 부재). 확정엔 '소형이라도 진짜 void 있는 샘플' 1개면 충분(kV60에서 잡는지 확인). 그 전까지 운영조건 kV60·R적정에서 거짓void=0(전 데이터 확인)이라 실무상 안전, False OK는 '미검증 한계'로 명시.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:H6"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>